<commit_message>
Small updates, working example with model reduction from 17 to 4.
</commit_message>
<xml_diff>
--- a/Comparison_linear_RMEP.xlsx
+++ b/Comparison_linear_RMEP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\MEP\RMEP_homotopy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE7F549-60FB-4829-84D3-5D2D08827377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A295134F-C410-434F-96A3-575AA51AC1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="612" yWindow="696" windowWidth="30384" windowHeight="17028" xr2:uid="{A4011660-FB7A-4DB9-A678-D73B0BBE67FE}"/>
+    <workbookView xWindow="30600" yWindow="-1944" windowWidth="33312" windowHeight="14532" activeTab="2" xr2:uid="{A4011660-FB7A-4DB9-A678-D73B0BBE67FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Times" sheetId="1" r:id="rId1"/>
@@ -409,7 +409,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -499,8 +499,6 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
@@ -1190,7 +1188,7 @@
       <c r="AI5" s="6">
         <v>2.8817240000000001E-2</v>
       </c>
-      <c r="AJ5" s="73" t="s">
+      <c r="AJ5" s="71" t="s">
         <v>65</v>
       </c>
       <c r="AK5" s="5">
@@ -1351,7 +1349,7 @@
       <c r="AE6" s="6">
         <v>0.11367843</v>
       </c>
-      <c r="AF6" s="71"/>
+      <c r="AF6" s="9"/>
       <c r="AG6" s="5">
         <v>0.26641277499999994</v>
       </c>
@@ -1361,7 +1359,7 @@
       <c r="AI6" s="6">
         <v>0.15541465500000001</v>
       </c>
-      <c r="AJ6" s="71"/>
+      <c r="AJ6" s="9"/>
       <c r="AK6" s="5">
         <v>0.34924788499999998</v>
       </c>
@@ -1478,7 +1476,7 @@
       <c r="AE7" s="5">
         <v>1.8763886000000003</v>
       </c>
-      <c r="AF7" s="71"/>
+      <c r="AF7" s="9"/>
       <c r="AG7" s="6">
         <v>1.1054329600000004</v>
       </c>
@@ -1488,7 +1486,7 @@
       <c r="AI7" s="5">
         <v>5.3976198599999998</v>
       </c>
-      <c r="AJ7" s="71"/>
+      <c r="AJ7" s="9"/>
       <c r="AK7" s="6">
         <v>1.73802514</v>
       </c>
@@ -1605,7 +1603,7 @@
       <c r="AE8" s="5">
         <v>32.783000000000001</v>
       </c>
-      <c r="AF8" s="71"/>
+      <c r="AF8" s="9"/>
       <c r="AG8" s="6">
         <v>4.0314480000000001</v>
       </c>
@@ -1615,7 +1613,7 @@
       <c r="AI8" s="5">
         <v>109.4554016</v>
       </c>
-      <c r="AJ8" s="71"/>
+      <c r="AJ8" s="9"/>
       <c r="AK8" s="6">
         <v>6.7989622000000001</v>
       </c>
@@ -1720,7 +1718,7 @@
       <c r="AE9" s="5">
         <v>658.49058000000002</v>
       </c>
-      <c r="AF9" s="71"/>
+      <c r="AF9" s="9"/>
       <c r="AG9" s="6">
         <v>12.6557928</v>
       </c>
@@ -1730,7 +1728,7 @@
       <c r="AI9" s="5">
         <v>2574.1812619000002</v>
       </c>
-      <c r="AJ9" s="71"/>
+      <c r="AJ9" s="9"/>
       <c r="AK9" s="6">
         <v>22.921736533333334</v>
       </c>
@@ -1826,7 +1824,6 @@
       <c r="AH10">
         <v>8008</v>
       </c>
-      <c r="AJ10" s="72"/>
       <c r="AK10" s="6">
         <v>67.346488899999997</v>
       </c>
@@ -3341,7 +3338,7 @@
     <col min="23" max="16384" width="8.88671875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" s="38" t="s">
         <v>23</v>
       </c>
@@ -3406,7 +3403,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="20">
         <v>2</v>
       </c>
@@ -3461,8 +3458,20 @@
       <c r="R2" s="27">
         <v>5.9272017089337676E-16</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="S2" s="69">
+        <v>1</v>
+      </c>
+      <c r="T2" s="69">
+        <v>1</v>
+      </c>
+      <c r="U2" s="67">
+        <v>1</v>
+      </c>
+      <c r="V2" s="67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="20">
         <v>2</v>
       </c>
@@ -3518,7 +3527,7 @@
         <v>5.2996279196627281E-16</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="20">
         <v>2</v>
       </c>
@@ -3574,7 +3583,7 @@
         <v>3.4933669516830488E-16</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="20">
         <v>2</v>
       </c>
@@ -3630,7 +3639,7 @@
         <v>4.4142888835188977E-16</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="20">
         <v>2</v>
       </c>
@@ -3686,7 +3695,7 @@
         <v>6.1218422523590752E-16</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="20">
         <v>2</v>
       </c>
@@ -3742,7 +3751,7 @@
         <v>5.9834603778956113E-16</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="20">
         <v>2</v>
       </c>
@@ -3798,7 +3807,7 @@
         <v>6.6948757332753836E-16</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="20">
         <v>2</v>
       </c>
@@ -3854,7 +3863,7 @@
         <v>1.4250195290242512E-15</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="20">
         <v>2</v>
       </c>
@@ -3910,7 +3919,7 @@
         <v>1.7643512804122316E-15</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="20">
         <v>2</v>
       </c>
@@ -3966,7 +3975,7 @@
         <v>1.5888123130548142E-15</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="20">
         <v>2</v>
       </c>
@@ -4022,7 +4031,7 @@
         <v>2.3356029560573503E-15</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="20">
         <v>2</v>
       </c>
@@ -4078,7 +4087,7 @@
         <v>3.6181620657799192E-15</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="20">
         <v>2</v>
       </c>
@@ -4134,7 +4143,7 @@
         <v>2.7838264868631072E-15</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="20">
         <v>2</v>
       </c>
@@ -4190,7 +4199,7 @@
         <v>7.3576942600163309E-15</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="20">
         <v>2</v>
       </c>

</xml_diff>